<commit_message>
added : Business based example files
</commit_message>
<xml_diff>
--- a/app/business/templates/other.xlsx
+++ b/app/business/templates/other.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="راهنما" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="products" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="راهنما" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'products'!$A$1:$G$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,23 +29,34 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Tahoma"/>
-      <b val="1"/>
-      <color rgb="002E86DE"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +65,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E86DE"/>
-        <bgColor rgb="002E86DE"/>
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,21 +108,50 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -444,112 +515,388 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📘 راهنمای فایل نمونه: سایر / فروشگاه عمومی</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+          <t>کد محصول</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>نام محصول</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>قیمت</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>موجودی</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>برند</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>توضیحات</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>لینک عکس</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>* اجباری</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>* اجباری</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>* اجباری</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>* اجباری</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>اختیاری</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>اختیاری</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>اختیاری</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>این فایل شامل چندین صفحه است:</t>
-        </is>
-      </c>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>PRD-001</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>رز هلندی دسته ۲۰ شاخه</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>گل‌فروشی بهار</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>تازه، مناسب هدیه</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>هر صفحه مخصوص یک دسته از محصولات شماست.</t>
-        </is>
-      </c>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>PRD-002</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>کتاب صد سال تنهایی</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>انتشارات نیلوفر</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>ترجمه فارسی، جلد سخت</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>PRD-003</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>عسل طبیعی یک کیلویی</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>420000</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>کندوی سبز</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>عسل آویشن کوهی، بدون افزودنی</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>📋 دسته‌های موجود:</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>PRD-004</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>جاشمعی سرامیکی دستساز</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>95000</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>کارگاه سفال</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>رنگ‌بندی متنوع، ارتفاع ۸ سانتی‌متر</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • 📦 محصولات عمومی  (صفحه: products)</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>PRD-005</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>چای ایرانی ۵۰۰ گرمی</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>145000</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>باغ چای لاهیجان</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>چای سر‌گل درجه یک لاهیجان</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>PRD-006</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>تابلو نقاشی آبرنگ</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>380000</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>گالری هنر نو</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>اثر هنری اصیل، ۳۰×۴۰ سانتی‌متر</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ نکات مهم:</t>
-        </is>
-      </c>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>PRD-007</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>ماگ سرامیکی طرح‌دار</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>75000</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>دیجی‌گیفت</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>ظرفیت ۳۵۰ میلی‌لیتر، ماشین‌شور</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>1. نام صفحه‌ها را تغییر ندهید</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>PRD-008</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>صابون طبیعی لوندر</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>55000</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>طبیعت‌گرا</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>صابون سرد، بدون مواد مصنوعی</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2. ردیف اول (نام ستون‌ها) را تغییر ندهید</t>
-        </is>
-      </c>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>PRD-009</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>ست قلم فلزی</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>220000</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>پن استار</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>ست ۵ عددی با جعبه هدیه</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>3. کد محصول باید یکتا باشد</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>4. فقط محصولاتی که دارید را وارد کنید</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>5. صفحه‌های خالی مشکلی ندارد (نادیده گرفته می‌شوند)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>💡 اگر یک دسته را ندارید، آن صفحه را خالی بگذارید</t>
-        </is>
-      </c>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>PRD-010</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>پادری پارچه‌ای</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>165000</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>خانه‌آرا</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>ضد لغزش، ابعاد ۶۰×۴۰ سانتی‌متر</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -557,55 +904,122 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0070AD47"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>بخش</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>توضیحات</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>کسب‌وکار</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>فروشگاه عمومی (سایر)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>ساختار فایل</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>این فایل دارای 1 شیت داده است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>شیت: products</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>لیست محصولات — برای هر نوع فروشگاهی قابل استفاده است</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>قیمت</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>عدد صحیح به تومان — بدون کاما یا متن</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>موجودی</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>عدد صحیح مثبت — ۰ به‌معنای ناموجود است</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>کد محصول</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>نام محصول</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>برند</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>قیمت</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>موجودی</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>توضیحات</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>باید منحصر‌به‌فرد باشد — تکراری موجب رونویسی می‌شود</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>لینک عکس</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>آدرس URL کامل عکس محصول (اختیاری)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>ردیف اول</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>ردیف اول هر شیت هدر است — تغییر ندهید</t>
         </is>
       </c>
     </row>

</xml_diff>